<commit_message>
adjust divide by 12 months
</commit_message>
<xml_diff>
--- a/wage.xlsx
+++ b/wage.xlsx
@@ -313,8 +313,8 @@
         <v>2400</v>
       </c>
       <c r="C3" s="1" t="n">
-        <f aca="false">B3*13</f>
-        <v>31200</v>
+        <f aca="false">B3*12</f>
+        <v>28800</v>
       </c>
       <c r="E3" s="1" t="n">
         <v>25</v>
@@ -324,8 +324,8 @@
         <v>4000</v>
       </c>
       <c r="G3" s="1" t="n">
-        <f aca="false">F3*13</f>
-        <v>52000</v>
+        <f aca="false">F3*12</f>
+        <v>48000</v>
       </c>
       <c r="H3" s="1" t="n">
         <f aca="false">F3*$H$1</f>
@@ -341,8 +341,8 @@
         <v>3200</v>
       </c>
       <c r="C4" s="1" t="n">
-        <f aca="false">B4*13</f>
-        <v>41600</v>
+        <f aca="false">B4*12</f>
+        <v>38400</v>
       </c>
       <c r="E4" s="1" t="n">
         <v>50</v>
@@ -352,8 +352,8 @@
         <v>8000</v>
       </c>
       <c r="G4" s="1" t="n">
-        <f aca="false">F4*13</f>
-        <v>104000</v>
+        <f aca="false">F4*12</f>
+        <v>96000</v>
       </c>
       <c r="H4" s="1" t="n">
         <f aca="false">F4*$H$1</f>
@@ -369,8 +369,8 @@
         <v>4000</v>
       </c>
       <c r="C5" s="1" t="n">
-        <f aca="false">B5*13</f>
-        <v>52000</v>
+        <f aca="false">B5*12</f>
+        <v>48000</v>
       </c>
       <c r="E5" s="1" t="n">
         <v>75</v>
@@ -380,8 +380,8 @@
         <v>12000</v>
       </c>
       <c r="G5" s="1" t="n">
-        <f aca="false">F5*13</f>
-        <v>156000</v>
+        <f aca="false">F5*12</f>
+        <v>144000</v>
       </c>
       <c r="H5" s="1" t="n">
         <f aca="false">F5*$H$1</f>
@@ -397,8 +397,8 @@
         <v>4800</v>
       </c>
       <c r="C6" s="1" t="n">
-        <f aca="false">B6*13</f>
-        <v>62400</v>
+        <f aca="false">B6*12</f>
+        <v>57600</v>
       </c>
       <c r="E6" s="1" t="n">
         <v>100</v>
@@ -408,8 +408,8 @@
         <v>16000</v>
       </c>
       <c r="G6" s="1" t="n">
-        <f aca="false">F6*13</f>
-        <v>208000</v>
+        <f aca="false">F6*12</f>
+        <v>192000</v>
       </c>
       <c r="H6" s="1" t="n">
         <f aca="false">F6*$H$1</f>
@@ -425,8 +425,8 @@
         <v>5600</v>
       </c>
       <c r="C7" s="1" t="n">
-        <f aca="false">B7*13</f>
-        <v>72800</v>
+        <f aca="false">B7*12</f>
+        <v>67200</v>
       </c>
       <c r="E7" s="1" t="n">
         <v>125</v>
@@ -436,8 +436,8 @@
         <v>20000</v>
       </c>
       <c r="G7" s="1" t="n">
-        <f aca="false">F7*13</f>
-        <v>260000</v>
+        <f aca="false">F7*12</f>
+        <v>240000</v>
       </c>
       <c r="H7" s="1" t="n">
         <f aca="false">F7*$H$1</f>
@@ -453,8 +453,8 @@
         <v>6400</v>
       </c>
       <c r="C8" s="1" t="n">
-        <f aca="false">B8*13</f>
-        <v>83200</v>
+        <f aca="false">B8*12</f>
+        <v>76800</v>
       </c>
       <c r="E8" s="1" t="n">
         <v>150</v>
@@ -464,8 +464,8 @@
         <v>24000</v>
       </c>
       <c r="G8" s="1" t="n">
-        <f aca="false">F8*13</f>
-        <v>312000</v>
+        <f aca="false">F8*12</f>
+        <v>288000</v>
       </c>
       <c r="H8" s="1" t="n">
         <f aca="false">F8*$H$1</f>
@@ -481,8 +481,8 @@
         <v>7200</v>
       </c>
       <c r="C9" s="1" t="n">
-        <f aca="false">B9*13</f>
-        <v>93600</v>
+        <f aca="false">B9*12</f>
+        <v>86400</v>
       </c>
       <c r="E9" s="1" t="n">
         <v>175</v>
@@ -492,8 +492,8 @@
         <v>28000</v>
       </c>
       <c r="G9" s="1" t="n">
-        <f aca="false">F9*13</f>
-        <v>364000</v>
+        <f aca="false">F9*12</f>
+        <v>336000</v>
       </c>
       <c r="H9" s="1" t="n">
         <f aca="false">F9*$H$1</f>
@@ -509,8 +509,8 @@
         <v>8000</v>
       </c>
       <c r="C10" s="1" t="n">
-        <f aca="false">B10*13</f>
-        <v>104000</v>
+        <f aca="false">B10*12</f>
+        <v>96000</v>
       </c>
       <c r="E10" s="1" t="n">
         <v>200</v>
@@ -520,8 +520,8 @@
         <v>32000</v>
       </c>
       <c r="G10" s="1" t="n">
-        <f aca="false">F10*13</f>
-        <v>416000</v>
+        <f aca="false">F10*12</f>
+        <v>384000</v>
       </c>
       <c r="H10" s="1" t="n">
         <f aca="false">F10*$H$1</f>
@@ -537,8 +537,8 @@
         <v>8800</v>
       </c>
       <c r="C11" s="1" t="n">
-        <f aca="false">B11*13</f>
-        <v>114400</v>
+        <f aca="false">B11*12</f>
+        <v>105600</v>
       </c>
       <c r="E11" s="1" t="n">
         <v>225</v>
@@ -548,8 +548,8 @@
         <v>36000</v>
       </c>
       <c r="G11" s="1" t="n">
-        <f aca="false">F11*13</f>
-        <v>468000</v>
+        <f aca="false">F11*12</f>
+        <v>432000</v>
       </c>
       <c r="H11" s="1" t="n">
         <f aca="false">F11*$H$1</f>
@@ -565,8 +565,8 @@
         <v>9600</v>
       </c>
       <c r="C12" s="1" t="n">
-        <f aca="false">B12*13</f>
-        <v>124800</v>
+        <f aca="false">B12*12</f>
+        <v>115200</v>
       </c>
       <c r="E12" s="1" t="n">
         <v>250</v>
@@ -576,8 +576,8 @@
         <v>40000</v>
       </c>
       <c r="G12" s="1" t="n">
-        <f aca="false">F12*13</f>
-        <v>520000</v>
+        <f aca="false">F12*12</f>
+        <v>480000</v>
       </c>
       <c r="H12" s="1" t="n">
         <f aca="false">F12*$H$1</f>
@@ -593,8 +593,8 @@
         <v>10400</v>
       </c>
       <c r="C13" s="1" t="n">
-        <f aca="false">B13*13</f>
-        <v>135200</v>
+        <f aca="false">B13*12</f>
+        <v>124800</v>
       </c>
       <c r="E13" s="1" t="n">
         <v>275</v>
@@ -604,8 +604,8 @@
         <v>44000</v>
       </c>
       <c r="G13" s="1" t="n">
-        <f aca="false">F13*13</f>
-        <v>572000</v>
+        <f aca="false">F13*12</f>
+        <v>528000</v>
       </c>
       <c r="H13" s="1" t="n">
         <f aca="false">F13*$H$1</f>
@@ -621,8 +621,8 @@
         <v>11200</v>
       </c>
       <c r="C14" s="1" t="n">
-        <f aca="false">B14*13</f>
-        <v>145600</v>
+        <f aca="false">B14*12</f>
+        <v>134400</v>
       </c>
       <c r="E14" s="1" t="n">
         <v>300</v>
@@ -632,8 +632,8 @@
         <v>48000</v>
       </c>
       <c r="G14" s="1" t="n">
-        <f aca="false">F14*13</f>
-        <v>624000</v>
+        <f aca="false">F14*12</f>
+        <v>576000</v>
       </c>
       <c r="H14" s="1" t="n">
         <f aca="false">F14*$H$1</f>
@@ -649,8 +649,8 @@
         <v>12000</v>
       </c>
       <c r="C15" s="1" t="n">
-        <f aca="false">B15*13</f>
-        <v>156000</v>
+        <f aca="false">B15*12</f>
+        <v>144000</v>
       </c>
       <c r="E15" s="1" t="n">
         <v>325</v>
@@ -660,8 +660,8 @@
         <v>52000</v>
       </c>
       <c r="G15" s="1" t="n">
-        <f aca="false">F15*13</f>
-        <v>676000</v>
+        <f aca="false">F15*12</f>
+        <v>624000</v>
       </c>
       <c r="H15" s="1" t="n">
         <f aca="false">F15*$H$1</f>
@@ -677,8 +677,8 @@
         <v>12800</v>
       </c>
       <c r="C16" s="1" t="n">
-        <f aca="false">B16*13</f>
-        <v>166400</v>
+        <f aca="false">B16*12</f>
+        <v>153600</v>
       </c>
       <c r="E16" s="1" t="n">
         <v>350</v>
@@ -688,8 +688,8 @@
         <v>56000</v>
       </c>
       <c r="G16" s="1" t="n">
-        <f aca="false">F16*13</f>
-        <v>728000</v>
+        <f aca="false">F16*12</f>
+        <v>672000</v>
       </c>
       <c r="H16" s="1" t="n">
         <f aca="false">F16*$H$1</f>
@@ -705,8 +705,8 @@
         <v>13600</v>
       </c>
       <c r="C17" s="1" t="n">
-        <f aca="false">B17*13</f>
-        <v>176800</v>
+        <f aca="false">B17*12</f>
+        <v>163200</v>
       </c>
       <c r="E17" s="1" t="n">
         <v>375</v>
@@ -716,8 +716,8 @@
         <v>60000</v>
       </c>
       <c r="G17" s="1" t="n">
-        <f aca="false">F17*13</f>
-        <v>780000</v>
+        <f aca="false">F17*12</f>
+        <v>720000</v>
       </c>
       <c r="H17" s="1" t="n">
         <f aca="false">F17*$H$1</f>
@@ -733,8 +733,8 @@
         <v>14400</v>
       </c>
       <c r="C18" s="1" t="n">
-        <f aca="false">B18*13</f>
-        <v>187200</v>
+        <f aca="false">B18*12</f>
+        <v>172800</v>
       </c>
       <c r="E18" s="1" t="n">
         <v>400</v>
@@ -744,8 +744,8 @@
         <v>64000</v>
       </c>
       <c r="G18" s="1" t="n">
-        <f aca="false">F18*13</f>
-        <v>832000</v>
+        <f aca="false">F18*12</f>
+        <v>768000</v>
       </c>
       <c r="H18" s="1" t="n">
         <f aca="false">F18*$H$1</f>
@@ -761,8 +761,8 @@
         <v>15200</v>
       </c>
       <c r="C19" s="1" t="n">
-        <f aca="false">B19*13</f>
-        <v>197600</v>
+        <f aca="false">B19*12</f>
+        <v>182400</v>
       </c>
       <c r="E19" s="1" t="n">
         <v>425</v>
@@ -772,8 +772,8 @@
         <v>68000</v>
       </c>
       <c r="G19" s="1" t="n">
-        <f aca="false">F19*13</f>
-        <v>884000</v>
+        <f aca="false">F19*12</f>
+        <v>816000</v>
       </c>
       <c r="H19" s="1" t="n">
         <f aca="false">F19*$H$1</f>
@@ -789,8 +789,8 @@
         <v>16000</v>
       </c>
       <c r="C20" s="1" t="n">
-        <f aca="false">B20*13</f>
-        <v>208000</v>
+        <f aca="false">B20*12</f>
+        <v>192000</v>
       </c>
       <c r="E20" s="1" t="n">
         <v>450</v>
@@ -800,8 +800,8 @@
         <v>72000</v>
       </c>
       <c r="G20" s="1" t="n">
-        <f aca="false">F20*13</f>
-        <v>936000</v>
+        <f aca="false">F20*12</f>
+        <v>864000</v>
       </c>
       <c r="H20" s="1" t="n">
         <f aca="false">F20*$H$1</f>
@@ -817,8 +817,8 @@
         <v>76000</v>
       </c>
       <c r="G21" s="1" t="n">
-        <f aca="false">F21*13</f>
-        <v>988000</v>
+        <f aca="false">F21*12</f>
+        <v>912000</v>
       </c>
       <c r="H21" s="1" t="n">
         <f aca="false">F21*$H$1</f>
@@ -834,8 +834,8 @@
         <v>80000</v>
       </c>
       <c r="G22" s="1" t="n">
-        <f aca="false">F22*13</f>
-        <v>1040000</v>
+        <f aca="false">F22*12</f>
+        <v>960000</v>
       </c>
       <c r="H22" s="1" t="n">
         <f aca="false">F22*$H$1</f>
@@ -851,8 +851,8 @@
         <v>84000</v>
       </c>
       <c r="G23" s="1" t="n">
-        <f aca="false">F23*13</f>
-        <v>1092000</v>
+        <f aca="false">F23*12</f>
+        <v>1008000</v>
       </c>
       <c r="H23" s="1" t="n">
         <f aca="false">F23*$H$1</f>
@@ -868,8 +868,8 @@
         <v>88000</v>
       </c>
       <c r="G24" s="1" t="n">
-        <f aca="false">F24*13</f>
-        <v>1144000</v>
+        <f aca="false">F24*12</f>
+        <v>1056000</v>
       </c>
       <c r="H24" s="1" t="n">
         <f aca="false">F24*$H$1</f>
@@ -885,8 +885,8 @@
         <v>92000</v>
       </c>
       <c r="G25" s="1" t="n">
-        <f aca="false">F25*13</f>
-        <v>1196000</v>
+        <f aca="false">F25*12</f>
+        <v>1104000</v>
       </c>
       <c r="H25" s="1" t="n">
         <f aca="false">F25*$H$1</f>
@@ -902,8 +902,8 @@
         <v>96000</v>
       </c>
       <c r="G26" s="1" t="n">
-        <f aca="false">F26*13</f>
-        <v>1248000</v>
+        <f aca="false">F26*12</f>
+        <v>1152000</v>
       </c>
       <c r="H26" s="1" t="n">
         <f aca="false">F26*$H$1</f>

</xml_diff>